<commit_message>
Atualização automática estagiários 2026-09-02 10:57
</commit_message>
<xml_diff>
--- a/de_para_orgao.xlsx
+++ b/de_para_orgao.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>SEE</t>
   </si>
@@ -127,13 +127,16 @@
   </si>
   <si>
     <t>sigla</t>
+  </si>
+  <si>
+    <t>NAO INFORMADO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -152,16 +155,28 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -178,11 +193,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDDDDDD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -192,6 +222,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -474,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -621,6 +654,14 @@
         <v>31</v>
       </c>
     </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>